<commit_message>
Add remaining shelf life, fix DIO variance decimals, update priority badge logic, align RCA/Store Action expiry rules
</commit_message>
<xml_diff>
--- a/data/sample/RCA_Rules.xlsx
+++ b/data/sample/RCA_Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8C3FD2-DF2C-49F6-94BD-ADDB19E36DD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626AB05E-2989-49CB-B176-0E772A023D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{71E9B6EE-C1E2-490E-8C11-E020BA23473F}"/>
   </bookViews>
@@ -99,13 +99,13 @@
     <t>If S09_Days_To_Season_End &lt;= S01_Weeks_Cover*7, then "Season-end write-off risk"</t>
   </si>
   <si>
-    <t>If S22_Shelf_Life_Remaining_Days &lt; S01_Weeks_Cover*7, then "Expiry Risk: Short-Expiry SKU ordered more than actual demand"</t>
-  </si>
-  <si>
     <t>First check for Root Cause Rule - 14, then rule - 15 amd then rule - 16 in that order. If rule-14 is true, do not check for rule-15 &amp; 16. If rule-15 is true, then do not check for rule-16</t>
   </si>
   <si>
     <t>If S01_Weeks_Cover &gt; 1.1 * S01_Weeks_Cover_Target AND no other rule fires, then "Monitor - Review at next weekly cycle"</t>
+  </si>
+  <si>
+    <t>If S22_Shelf_Life_Remaining_Days &lt;= S01_Weeks_Cover*7, then "Expiry Risk: Short-Expiry SKU ordered more than actual demand"</t>
   </si>
 </sst>
 </file>
@@ -594,7 +594,7 @@
         <v>5</v>
       </c>
       <c r="N15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -602,7 +602,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="N16" t="s">
         <v>4</v>
@@ -640,7 +640,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>